<commit_message>
Fix màn hình Quản lý Hệ thống VTS, Quản lý Trạm Radar, Báo cáo [F-158] Biểu 11-N: Thống kê về hệ thống giám sát và điều phối giao thông hàng hải (VTS)
</commit_message>
<xml_diff>
--- a/src/main/resources/public/template_export/BCKCHT_168.xlsx
+++ b/src/main/resources/public/template_export/BCKCHT_168.xlsx
@@ -226,9 +226,6 @@
     <t>${entry.value[0].ghiChu.asText()}</t>
   </si>
   <si>
-    <t>${thiz.getCateOtherText('DM_APP_PARAM',entry.key, 'LOAI_KCHT')}</t>
-  </si>
-  <si>
     <t xml:space="preserve">Đơn vị báo cáo: </t>
   </si>
   <si>
@@ -250,16 +247,19 @@
     <t>${idx1+1}</t>
   </si>
   <si>
-    <t>${thiz.getCateOtherText('DM_APP_PARAM',item.nhom.asText(), 'LOAI_KCHT')} ${item.tenDiemNeo.asText()}</t>
-  </si>
-  <si>
-    <t>${thiz.getCateOtherText('KCHT_CB',table.key, 'CB')}</t>
-  </si>
-  <si>
     <t>${entry.value[0].viTriKhu.asText()}</t>
   </si>
   <si>
     <t>${item.viTriDiemNeo.asText()}</t>
+  </si>
+  <si>
+    <t>${this.getCateOtherText('DM_APP_PARAM',entry.key, 'LOAI_KCHT')}</t>
+  </si>
+  <si>
+    <t>${this.getCateOtherText('KCHT_CB',table.key, 'CB')}</t>
+  </si>
+  <si>
+    <t>${this.getCateOtherText('DM_APP_PARAM',item.nhom.asText(), 'LOAI_KCHT')} ${item.tenDiemNeo.asText()}</t>
   </si>
 </sst>
 </file>
@@ -463,6 +463,18 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
@@ -492,18 +504,6 @@
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -784,12 +784,12 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:L19"/>
-  <sheetFormatPr defaultRowHeight="12.75" ns2:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="5.85546875" style="1" customWidth="1"/>
     <col min="2" max="2" width="46.28515625" style="1" customWidth="1"/>
@@ -802,139 +802,139 @@
     <col min="13" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ns2:dyDescent="0.2">
-      <c r="A1" s="27" t="s">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A1" s="31" t="s">
         <v>14</v>
       </c>
-      <c r="B1" s="28"/>
+      <c r="B1" s="32"/>
       <c r="C1" s="9"/>
       <c r="D1" s="20"/>
       <c r="E1" s="9"/>
       <c r="F1" s="9"/>
       <c r="G1" s="9"/>
-      <c r="I1" s="23" t="s">
-        <v>34</v>
-      </c>
-      <c r="J1" s="23"/>
-      <c r="K1" s="23"/>
-      <c r="L1" s="23"/>
-    </row>
-    <row r="2" spans="1:12" ns2:dyDescent="0.2">
-      <c r="A2" s="28" t="s">
+      <c r="I1" s="27" t="s">
+        <v>33</v>
+      </c>
+      <c r="J1" s="27"/>
+      <c r="K1" s="27"/>
+      <c r="L1" s="27"/>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A2" s="32" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="27"/>
+      <c r="B2" s="31"/>
       <c r="C2" s="8"/>
       <c r="D2" s="19"/>
       <c r="E2" s="8"/>
       <c r="F2" s="8"/>
       <c r="G2" s="8"/>
-      <c r="I2" s="28" t="s">
-        <v>35</v>
-      </c>
-      <c r="J2" s="28"/>
-      <c r="K2" s="28"/>
-      <c r="L2" s="28"/>
-    </row>
-    <row r="3" spans="1:12" ht="12.75" customHeight="1" ns2:dyDescent="0.2">
-      <c r="A3" s="28" t="s">
+      <c r="I2" s="32" t="s">
+        <v>34</v>
+      </c>
+      <c r="J2" s="32"/>
+      <c r="K2" s="32"/>
+      <c r="L2" s="32"/>
+    </row>
+    <row r="3" spans="1:12" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="32" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="28"/>
+      <c r="B3" s="32"/>
       <c r="C3" s="9"/>
       <c r="D3" s="20"/>
       <c r="E3" s="9"/>
       <c r="F3" s="9"/>
       <c r="G3" s="9"/>
-      <c r="I3" s="24" t="s">
+      <c r="I3" s="28" t="s">
+        <v>36</v>
+      </c>
+      <c r="J3" s="28"/>
+      <c r="K3" s="28"/>
+      <c r="L3" s="28"/>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="I4" s="36" t="s">
+        <v>35</v>
+      </c>
+      <c r="J4" s="36"/>
+      <c r="K4" s="36"/>
+      <c r="L4" s="36"/>
+    </row>
+    <row r="5" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="33" t="s">
+        <v>23</v>
+      </c>
+      <c r="B5" s="33"/>
+      <c r="C5" s="33"/>
+      <c r="D5" s="33"/>
+      <c r="E5" s="33"/>
+      <c r="F5" s="33"/>
+      <c r="G5" s="33"/>
+      <c r="H5" s="33"/>
+      <c r="I5" s="33"/>
+      <c r="J5" s="33"/>
+      <c r="K5" s="33"/>
+    </row>
+    <row r="6" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A6" s="34" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" s="34"/>
+      <c r="C6" s="34"/>
+      <c r="D6" s="34"/>
+      <c r="E6" s="34"/>
+      <c r="F6" s="34"/>
+      <c r="G6" s="34"/>
+      <c r="H6" s="34"/>
+      <c r="I6" s="34"/>
+      <c r="J6" s="34"/>
+      <c r="K6" s="34"/>
+    </row>
+    <row r="8" spans="1:12" s="2" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="26" t="s">
+        <v>0</v>
+      </c>
+      <c r="B8" s="26" t="s">
+        <v>10</v>
+      </c>
+      <c r="C8" s="29" t="s">
         <v>37</v>
       </c>
-      <c r="J3" s="24"/>
-      <c r="K3" s="24"/>
-      <c r="L3" s="24"/>
-    </row>
-    <row r="4" spans="1:12" ns2:dyDescent="0.2">
-      <c r="I4" s="32" t="s">
-        <v>36</v>
-      </c>
-      <c r="J4" s="32"/>
-      <c r="K4" s="32"/>
-      <c r="L4" s="32"/>
-    </row>
-    <row r="5" spans="1:12" ht="15.75" customHeight="1" ns2:dyDescent="0.2">
-      <c r="A5" s="29" t="s">
-        <v>23</v>
-      </c>
-      <c r="B5" s="29"/>
-      <c r="C5" s="29"/>
-      <c r="D5" s="29"/>
-      <c r="E5" s="29"/>
-      <c r="F5" s="29"/>
-      <c r="G5" s="29"/>
-      <c r="H5" s="29"/>
-      <c r="I5" s="29"/>
-      <c r="J5" s="29"/>
-      <c r="K5" s="29"/>
-    </row>
-    <row r="6" spans="1:12" ht="15.75" ns2:dyDescent="0.25">
-      <c r="A6" s="30" t="s">
-        <v>9</v>
-      </c>
-      <c r="B6" s="30"/>
-      <c r="C6" s="30"/>
-      <c r="D6" s="30"/>
-      <c r="E6" s="30"/>
-      <c r="F6" s="30"/>
-      <c r="G6" s="30"/>
-      <c r="H6" s="30"/>
-      <c r="I6" s="30"/>
-      <c r="J6" s="30"/>
-      <c r="K6" s="30"/>
-    </row>
-    <row r="8" spans="1:12" s="2" customFormat="1" ht="22.5" customHeight="1" ns2:dyDescent="0.2">
-      <c r="A8" s="36" t="s">
-        <v>0</v>
-      </c>
-      <c r="B8" s="36" t="s">
-        <v>10</v>
-      </c>
-      <c r="C8" s="25" t="s">
-        <v>38</v>
-      </c>
-      <c r="D8" s="36" t="s">
+      <c r="D8" s="26" t="s">
         <v>24</v>
       </c>
-      <c r="E8" s="36"/>
-      <c r="F8" s="25" t="s">
+      <c r="E8" s="26"/>
+      <c r="F8" s="29" t="s">
         <v>17</v>
       </c>
-      <c r="G8" s="25" t="s">
+      <c r="G8" s="29" t="s">
         <v>18</v>
       </c>
-      <c r="H8" s="36" t="s">
+      <c r="H8" s="26" t="s">
         <v>19</v>
       </c>
-      <c r="I8" s="36"/>
-      <c r="J8" s="36" t="s">
+      <c r="I8" s="26"/>
+      <c r="J8" s="26" t="s">
         <v>11</v>
       </c>
-      <c r="K8" s="36"/>
-      <c r="L8" s="25" t="s">
+      <c r="K8" s="26"/>
+      <c r="L8" s="29" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="9" spans="1:12" s="2" customFormat="1" ht="35.25" customHeight="1" ns2:dyDescent="0.2">
-      <c r="A9" s="36"/>
-      <c r="B9" s="36"/>
-      <c r="C9" s="26"/>
+    <row r="9" spans="1:12" s="2" customFormat="1" ht="35.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A9" s="26"/>
+      <c r="B9" s="26"/>
+      <c r="C9" s="30"/>
       <c r="D9" s="21" t="s">
         <v>15</v>
       </c>
       <c r="E9" s="21" t="s">
         <v>16</v>
       </c>
-      <c r="F9" s="26"/>
-      <c r="G9" s="26"/>
+      <c r="F9" s="30"/>
+      <c r="G9" s="30"/>
       <c r="H9" s="16" t="s">
         <v>21</v>
       </c>
@@ -947,9 +947,9 @@
       <c r="K9" s="16" t="s">
         <v>20</v>
       </c>
-      <c r="L9" s="31"/>
-    </row>
-    <row r="10" spans="1:12" s="3" customFormat="1" ns2:dyDescent="0.2">
+      <c r="L9" s="35"/>
+    </row>
+    <row r="10" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A10" s="15" t="s">
         <v>1</v>
       </c>
@@ -987,12 +987,12 @@
         <v>10</v>
       </c>
     </row>
-    <row r="11" spans="1:12" ht="16.5" customHeight="1" ns2:dyDescent="0.2">
+    <row r="11" spans="1:12" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="4" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B11" s="12" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C11" s="12"/>
       <c r="D11" s="12"/>
@@ -1005,13 +1005,13 @@
       <c r="K11" s="7"/>
       <c r="L11" s="7"/>
     </row>
-    <row r="12" spans="1:12" ht="39.950000000000003" customHeight="1" ns2:dyDescent="0.2">
+    <row r="12" spans="1:12" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="4"/>
       <c r="B12" s="12" t="s">
-        <v>33</v>
+        <v>42</v>
       </c>
       <c r="C12" s="22" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="D12" s="22" t="s">
         <v>25</v>
@@ -1023,7 +1023,7 @@
         <v>27</v>
       </c>
       <c r="G12" s="22" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="H12" s="22" t="s">
         <v>28</v>
@@ -1041,13 +1041,13 @@
         <v>32</v>
       </c>
     </row>
-    <row r="13" spans="1:12" ht="39.950000000000003" customHeight="1" ns2:dyDescent="0.2">
+    <row r="13" spans="1:12" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="5"/>
       <c r="B13" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="C13" s="22" t="s">
         <v>41</v>
-      </c>
-      <c r="C13" s="22" t="s">
-        <v>44</v>
       </c>
       <c r="D13" s="22"/>
       <c r="E13" s="22"/>
@@ -1059,90 +1059,81 @@
       <c r="K13" s="22"/>
       <c r="L13" s="22"/>
     </row>
-    <row r="15" spans="1:12" ns2:dyDescent="0.2">
-      <c r="A15" s="34" t="s">
+    <row r="15" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A15" s="24" t="s">
         <v>5</v>
       </c>
-      <c r="B15" s="35"/>
+      <c r="B15" s="25"/>
       <c r="C15" s="11"/>
       <c r="D15" s="18"/>
       <c r="E15" s="11"/>
       <c r="F15" s="11"/>
       <c r="G15" s="11"/>
-      <c r="H15" s="34" t="s">
+      <c r="H15" s="24" t="s">
         <v>7</v>
       </c>
-      <c r="I15" s="35"/>
-      <c r="J15" s="35"/>
-      <c r="K15" s="35"/>
-    </row>
-    <row r="16" spans="1:12" ns2:dyDescent="0.2">
-      <c r="A16" s="33" t="s">
+      <c r="I15" s="25"/>
+      <c r="J15" s="25"/>
+      <c r="K15" s="25"/>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A16" s="23" t="s">
         <v>6</v>
       </c>
-      <c r="B16" s="33"/>
+      <c r="B16" s="23"/>
       <c r="C16" s="10"/>
       <c r="D16" s="17"/>
       <c r="E16" s="10"/>
       <c r="F16" s="10"/>
       <c r="G16" s="10"/>
-      <c r="H16" s="33" t="s">
+      <c r="H16" s="23" t="s">
         <v>8</v>
       </c>
-      <c r="I16" s="33"/>
-      <c r="J16" s="33"/>
-      <c r="K16" s="33"/>
-    </row>
-    <row r="17" spans="1:11" ns2:dyDescent="0.2">
-      <c r="A17" s="33"/>
-      <c r="B17" s="33"/>
+      <c r="I16" s="23"/>
+      <c r="J16" s="23"/>
+      <c r="K16" s="23"/>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A17" s="23"/>
+      <c r="B17" s="23"/>
       <c r="C17" s="10"/>
       <c r="D17" s="17"/>
       <c r="E17" s="10"/>
       <c r="F17" s="10"/>
       <c r="G17" s="10"/>
-      <c r="H17" s="33"/>
-      <c r="I17" s="33"/>
-      <c r="J17" s="33"/>
-      <c r="K17" s="33"/>
-    </row>
-    <row r="18" spans="1:11" ns2:dyDescent="0.2">
-      <c r="A18" s="33"/>
-      <c r="B18" s="33"/>
+      <c r="H17" s="23"/>
+      <c r="I17" s="23"/>
+      <c r="J17" s="23"/>
+      <c r="K17" s="23"/>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A18" s="23"/>
+      <c r="B18" s="23"/>
       <c r="C18" s="10"/>
       <c r="D18" s="17"/>
       <c r="E18" s="10"/>
       <c r="F18" s="10"/>
       <c r="G18" s="10"/>
-      <c r="H18" s="33"/>
-      <c r="I18" s="33"/>
-      <c r="J18" s="33"/>
-      <c r="K18" s="33"/>
-    </row>
-    <row r="19" spans="1:11" ns2:dyDescent="0.2">
-      <c r="A19" s="33"/>
-      <c r="B19" s="33"/>
+      <c r="H18" s="23"/>
+      <c r="I18" s="23"/>
+      <c r="J18" s="23"/>
+      <c r="K18" s="23"/>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A19" s="23"/>
+      <c r="B19" s="23"/>
       <c r="C19" s="10"/>
       <c r="D19" s="17"/>
       <c r="E19" s="10"/>
       <c r="F19" s="10"/>
       <c r="G19" s="10"/>
-      <c r="H19" s="33"/>
-      <c r="I19" s="33"/>
-      <c r="J19" s="33"/>
-      <c r="K19" s="33"/>
+      <c r="H19" s="23"/>
+      <c r="I19" s="23"/>
+      <c r="J19" s="23"/>
+      <c r="K19" s="23"/>
     </row>
   </sheetData>
   <mergeCells count="22">
-    <mergeCell ref="H16:K19"/>
-    <mergeCell ref="A16:B19"/>
-    <mergeCell ref="A15:B15"/>
-    <mergeCell ref="H15:K15"/>
-    <mergeCell ref="J8:K8"/>
-    <mergeCell ref="A8:A9"/>
-    <mergeCell ref="B8:B9"/>
-    <mergeCell ref="D8:E8"/>
-    <mergeCell ref="H8:I8"/>
     <mergeCell ref="I1:L1"/>
     <mergeCell ref="I3:L3"/>
     <mergeCell ref="F8:F9"/>
@@ -1156,9 +1147,18 @@
     <mergeCell ref="C8:C9"/>
     <mergeCell ref="I2:L2"/>
     <mergeCell ref="I4:L4"/>
+    <mergeCell ref="H16:K19"/>
+    <mergeCell ref="A16:B19"/>
+    <mergeCell ref="A15:B15"/>
+    <mergeCell ref="H15:K15"/>
+    <mergeCell ref="J8:K8"/>
+    <mergeCell ref="A8:A9"/>
+    <mergeCell ref="B8:B9"/>
+    <mergeCell ref="D8:E8"/>
+    <mergeCell ref="H8:I8"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="3" fitToWidth="1" fitToHeight="0" orientation="landscape" r:id="rId1"/>
+  <pageSetup paperSize="3" fitToHeight="0" orientation="landscape" r:id="rId1"/>
   <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>